<commit_message>
Conso > achats : refonte complète (réponse aux exemples du fisc)
Répond exemple par exemple via le mapping caisse↔facture↔inventaire, achats nets
des avoirs vs conso mesurée, par exercice, sans supposition :
- Haute Côte de Beaune : le « 12 950 cl de blanc sans achat » est une confusion
  de couleur (blanc réel = 450 cl ; le volume visé = rouge, acheté 202 L ≥ conso
  172 L ; Nuits blanc = vin distinct, acheté).
- Eaux-de-vie / liqueurs / Martini : achats existent sous libellés frères
  (FRAMBOISE SAUVAGE, MIRABELLE, POIRE WILLIAM, MARTINI BIANCO) → achat ≥ conso.
- Calvados : seul écart, entièrement en estimation de cuisson (flambés) ; la
  caisse ne vend que 1,4 L au verre. Alcool de cuisine = coût, pas vente.
- Bilan matière global : +3 048 L net (excédent).
- 7 chapitres, 5 XLSX (un par section). Ancien XLSX orphelin supprimé.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/RF-coefficients-de-revente.xlsx
+++ b/public/documents/pieces-defense/RF-coefficients-de-revente.xlsx
@@ -504,13 +504,13 @@
         <v>3.54</v>
       </c>
       <c r="F2" t="n">
-        <v>0.224</v>
+        <v>0.26</v>
       </c>
       <c r="G2" t="n">
-        <v>226553</v>
+        <v>215973</v>
       </c>
       <c r="H2" t="n">
-        <v>2.74</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="3">
@@ -532,13 +532,13 @@
         <v>3.83</v>
       </c>
       <c r="F3" t="n">
-        <v>0.224</v>
+        <v>0.26</v>
       </c>
       <c r="G3" t="n">
-        <v>30616</v>
+        <v>29186</v>
       </c>
       <c r="H3" t="n">
-        <v>2.97</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="4">
@@ -560,13 +560,13 @@
         <v>7.43</v>
       </c>
       <c r="F4" t="n">
-        <v>0.224</v>
+        <v>0.26</v>
       </c>
       <c r="G4" t="n">
-        <v>36354</v>
+        <v>34656</v>
       </c>
       <c r="H4" t="n">
-        <v>5.76</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="5">
@@ -588,13 +588,13 @@
         <v>3.97</v>
       </c>
       <c r="F5" t="n">
-        <v>0.224</v>
+        <v>0.26</v>
       </c>
       <c r="G5" t="n">
-        <v>7446</v>
+        <v>7098</v>
       </c>
       <c r="H5" t="n">
-        <v>3.08</v>
+        <v>2.93</v>
       </c>
     </row>
     <row r="6">
@@ -616,13 +616,13 @@
         <v>3.82</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.224</v>
+        <v>0.26</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>300969</v>
+        <v>286914</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>2.96</v>
+        <v>2.82</v>
       </c>
     </row>
   </sheetData>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -778,14 +778,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sur-versement au verre et cocktails (free-pour, Kerr 2008)</t>
+          <t>Sur-versement vins/spiritueux/cocktails (free-pour : Kerr 2008, Wansink 2005)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>807</v>
+        <v>1058</v>
       </c>
       <c r="C8" t="n">
-        <v>0.076</v>
+        <v>0.1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Degustation offerte (pichet + vin nomme au verre)</t>
+          <t>Degustation offerte (note par note, annexe C)</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -818,10 +818,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>126</v>
+        <v>260</v>
       </c>
       <c r="C10" t="n">
-        <v>0.012</v>
+        <v>0.024</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -832,14 +832,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Freinte technique de la biere pression (mousse, lignes)</t>
+          <t>Cremant sur-versé (free-pour +23,6 %)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="C11" t="n">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -850,48 +850,66 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Freinte technique de la biere pression (mousse, lignes)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>129</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NON</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Stock final (inventaire)</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B13" t="n">
         <v>213</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C13" t="n">
         <v>0.02</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>NON</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL conso + stock</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>8945</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>0.842</v>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>TOTAL conso + stock</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>9417</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Achats d'alcool (référence)</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>10622</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>